<commit_message>
Golden 50: workbook with Jack's draft carried over; course file restored
Jack's own evidence_quote, entities and needs_review are copied into editable cells;
his free-form topic/intent/severity/sentiment sit in locked my_draft_* columns. The
contract topic/intent/severity/sentiment cells stay blank for him to pick. His draft is
saved as evals/golden/jack_draft_freeform_labels.csv. data/golden_50_to_label.csv
(git-ignored) restored byte-exact to the course manifest checksum.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evals/golden_50_labels.xlsx
+++ b/evals/golden_50_labels.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,8 +33,12 @@
     <font>
       <name val="Arial"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -48,7 +52,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,14 +78,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -441,22 +463,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="64" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,52 +504,77 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>my_draft_topic</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>my_draft_intent</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>my_draft_severity</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>my_draft_sentiment</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>topic</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>intent</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>sentiment</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>evidence_quote</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>needs_review</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ambiguous</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>accepted_alternatives</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>check_quote_in_text</t>
         </is>
       </c>
     </row>
@@ -540,16 +592,53 @@
       <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr"/>
-      <c r="K2" s="3" t="inlineStr"/>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>content_moderation</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr"/>
+      <c r="I2" s="4" t="inlineStr"/>
+      <c r="J2" s="4" t="inlineStr"/>
+      <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; Christian music; conservative music; LGBTQ+ pride</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>Banning conservative music that speaks truth</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr"/>
+      <c r="P2" s="4" t="inlineStr"/>
+      <c r="Q2" s="4" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -565,16 +654,53 @@
       <c r="C3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Great app use it every chance I get</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr"/>
+      <c r="P3" s="4" t="inlineStr"/>
+      <c r="Q3" s="4" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -590,16 +716,53 @@
       <c r="C4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>It's really an amazing experience with Spotify</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr"/>
+      <c r="P4" s="4" t="inlineStr"/>
+      <c r="Q4" s="4" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -615,16 +778,53 @@
       <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr"/>
-      <c r="M5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>ads; free_tier_limitations</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; ads; app functionality</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>limited functionality..it's just too much</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr"/>
+      <c r="P5" s="4" t="inlineStr"/>
+      <c r="Q5" s="4" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -640,16 +840,53 @@
       <c r="C6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr"/>
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>I just loved it</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr"/>
+      <c r="P6" s="4" t="inlineStr"/>
+      <c r="Q6" s="4" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -665,16 +902,53 @@
       <c r="C7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>general_dissatisfaction</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Hate this application</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr"/>
+      <c r="P7" s="4" t="inlineStr"/>
+      <c r="Q7" s="4" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -690,16 +964,53 @@
       <c r="C8" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr"/>
+      <c r="P8" s="4" t="inlineStr"/>
+      <c r="Q8" s="4" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -715,16 +1026,53 @@
       <c r="C9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr"/>
+      <c r="P9" s="4" t="inlineStr"/>
+      <c r="Q9" s="4" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -740,16 +1088,53 @@
       <c r="C10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="3" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>content_diversity</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>very diverse</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr"/>
+      <c r="P10" s="4" t="inlineStr"/>
+      <c r="Q10" s="4" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -765,16 +1150,53 @@
       <c r="C11" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
-      <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>subscription; ads</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; Duo Premium</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>No ads at all!</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr"/>
+      <c r="P11" s="4" t="inlineStr"/>
+      <c r="Q11" s="4" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -790,16 +1212,53 @@
       <c r="C12" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>playback</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>bug_report</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; music playback</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>it o ly plays a little bit then it stops</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr"/>
+      <c r="P12" s="4" t="inlineStr"/>
+      <c r="Q12" s="4" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -815,16 +1274,53 @@
       <c r="C13" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>app_stability</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>support_resolution</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; Spotify Support; Sarah</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>I was able to get the app working again</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr"/>
+      <c r="P13" s="4" t="inlineStr"/>
+      <c r="Q13" s="4" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -840,16 +1336,53 @@
       <c r="C14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr"/>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>general_dissatisfaction</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>This app is bad work</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr"/>
+      <c r="P14" s="4" t="inlineStr"/>
+      <c r="Q14" s="4" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -865,16 +1398,53 @@
       <c r="C15" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Great</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr"/>
+      <c r="P15" s="4" t="inlineStr"/>
+      <c r="Q15" s="4" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -890,16 +1460,53 @@
       <c r="C16" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="3" t="inlineStr"/>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
-      <c r="J16" s="3" t="inlineStr"/>
-      <c r="K16" s="3" t="inlineStr"/>
-      <c r="L16" s="3" t="inlineStr"/>
-      <c r="M16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="inlineStr"/>
+      <c r="Q16" s="4" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -915,16 +1522,53 @@
       <c r="C17" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr"/>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr"/>
-      <c r="J17" s="3" t="inlineStr"/>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>ads</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>mixed_feedback</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; music; ads</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>I like it but god I hate it when the music Interrupts my ads</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr"/>
+      <c r="P17" s="4" t="inlineStr"/>
+      <c r="Q17" s="4" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -940,16 +1584,53 @@
       <c r="C18" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr"/>
-      <c r="K18" s="3" t="inlineStr"/>
-      <c r="L18" s="3" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>music_catalog</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Lhat ng song nasa spotify</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr"/>
+      <c r="P18" s="4" t="inlineStr"/>
+      <c r="Q18" s="4" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -965,16 +1646,53 @@
       <c r="C19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr"/>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="3" t="inlineStr"/>
-      <c r="K19" s="3" t="inlineStr"/>
-      <c r="L19" s="3" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Avtar sungh</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr"/>
+      <c r="P19" s="4" t="inlineStr"/>
+      <c r="Q19" s="4" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -990,16 +1708,53 @@
       <c r="C20" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr"/>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="3" t="inlineStr"/>
-      <c r="K20" s="3" t="inlineStr"/>
-      <c r="L20" s="3" t="inlineStr"/>
-      <c r="M20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>lyrics</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>bug_report</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; lyrics</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>lirik nya kdang gaada</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="inlineStr"/>
+      <c r="Q20" s="4" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1015,16 +1770,53 @@
       <c r="C21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr"/>
-      <c r="J21" s="3" t="inlineStr"/>
-      <c r="K21" s="3" t="inlineStr"/>
-      <c r="L21" s="3" t="inlineStr"/>
-      <c r="M21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>general_dissatisfaction</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr"/>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Hate This application</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr"/>
+      <c r="P21" s="4" t="inlineStr"/>
+      <c r="Q21" s="4" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1040,16 +1832,53 @@
       <c r="C22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="3" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr"/>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr"/>
-      <c r="J22" s="3" t="inlineStr"/>
-      <c r="K22" s="3" t="inlineStr"/>
-      <c r="L22" s="3" t="inlineStr"/>
-      <c r="M22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>boycott; political_or_religious_protest</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>boycott</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
+      <c r="I22" s="4" t="inlineStr"/>
+      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; Sweden; Qur'an</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>We are boycotting Swedish app</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr"/>
+      <c r="P22" s="4" t="inlineStr"/>
+      <c r="Q22" s="4" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1065,16 +1894,53 @@
       <c r="C23" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr"/>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr"/>
-      <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr"/>
-      <c r="M23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>recommendations; playlists</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; playlists; recommendations</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Spotify gave me recommendations for an AWESOME Playlist</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr"/>
+      <c r="P23" s="4" t="inlineStr"/>
+      <c r="Q23" s="4" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1090,16 +1956,53 @@
       <c r="C24" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D24" s="3" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr"/>
-      <c r="G24" s="3" t="inlineStr"/>
-      <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr"/>
-      <c r="J24" s="3" t="inlineStr"/>
-      <c r="K24" s="3" t="inlineStr"/>
-      <c r="L24" s="3" t="inlineStr"/>
-      <c r="M24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>one of the best Music Apps</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr"/>
+      <c r="P24" s="4" t="inlineStr"/>
+      <c r="Q24" s="4" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1115,16 +2018,53 @@
       <c r="C25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr"/>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr"/>
-      <c r="J25" s="3" t="inlineStr"/>
-      <c r="K25" s="3" t="inlineStr"/>
-      <c r="L25" s="3" t="inlineStr"/>
-      <c r="M25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>ads</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; ads</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>harr ek song ke baad ad</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="inlineStr"/>
+      <c r="P25" s="4" t="inlineStr"/>
+      <c r="Q25" s="4" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1140,16 +2080,53 @@
       <c r="C26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="3" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr"/>
-      <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr"/>
-      <c r="I26" s="3" t="inlineStr"/>
-      <c r="J26" s="3" t="inlineStr"/>
-      <c r="K26" s="3" t="inlineStr"/>
-      <c r="L26" s="3" t="inlineStr"/>
-      <c r="M26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>app_update; playback</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>bug_report</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr"/>
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; updates; playback</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>we cannot playback the songs</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr"/>
+      <c r="P26" s="4" t="inlineStr"/>
+      <c r="Q26" s="4" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1165,16 +2142,53 @@
       <c r="C27" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr"/>
-      <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr"/>
-      <c r="J27" s="3" t="inlineStr"/>
-      <c r="K27" s="3" t="inlineStr"/>
-      <c r="L27" s="3" t="inlineStr"/>
-      <c r="M27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>Awesomeness</t>
+        </is>
+      </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="inlineStr"/>
+      <c r="P27" s="4" t="inlineStr"/>
+      <c r="Q27" s="4" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1190,16 +2204,53 @@
       <c r="C28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr"/>
-      <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="3" t="inlineStr"/>
-      <c r="L28" s="3" t="inlineStr"/>
-      <c r="M28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr"/>
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>Bheekhmangon</t>
+        </is>
+      </c>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr"/>
+      <c r="P28" s="4" t="inlineStr"/>
+      <c r="Q28" s="4" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1215,16 +2266,53 @@
       <c r="C29" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="3" t="inlineStr"/>
-      <c r="I29" s="3" t="inlineStr"/>
-      <c r="J29" s="3" t="inlineStr"/>
-      <c r="K29" s="3" t="inlineStr"/>
-      <c r="L29" s="3" t="inlineStr"/>
-      <c r="M29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>music_content</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr"/>
+      <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr"/>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; Stoli Canales; Unconditional Love</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>Unconditional love, Stoli Canales</t>
+        </is>
+      </c>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr"/>
+      <c r="P29" s="4" t="inlineStr"/>
+      <c r="Q29" s="4" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1240,16 +2328,53 @@
       <c r="C30" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="3" t="inlineStr"/>
-      <c r="G30" s="3" t="inlineStr"/>
-      <c r="H30" s="3" t="inlineStr"/>
-      <c r="I30" s="3" t="inlineStr"/>
-      <c r="J30" s="3" t="inlineStr"/>
-      <c r="K30" s="3" t="inlineStr"/>
-      <c r="L30" s="3" t="inlineStr"/>
-      <c r="M30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>free_tier_limitations; playback_controls; app_update</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr"/>
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr"/>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; Premium; shuffle; playback controls</t>
+        </is>
+      </c>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>we can't CHOOSE song after a song played</t>
+        </is>
+      </c>
+      <c r="N30" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr"/>
+      <c r="P30" s="4" t="inlineStr"/>
+      <c r="Q30" s="4" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1265,16 +2390,53 @@
       <c r="C31" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr"/>
-      <c r="G31" s="3" t="inlineStr"/>
-      <c r="H31" s="3" t="inlineStr"/>
-      <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="inlineStr"/>
-      <c r="K31" s="3" t="inlineStr"/>
-      <c r="L31" s="3" t="inlineStr"/>
-      <c r="M31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>pricing; free_tier_limitations</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; Premium</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>everything basic features is premium</t>
+        </is>
+      </c>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr"/>
+      <c r="P31" s="4" t="inlineStr"/>
+      <c r="Q31" s="4" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1290,16 +2452,53 @@
       <c r="C32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D32" s="3" t="inlineStr"/>
-      <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr"/>
-      <c r="G32" s="3" t="inlineStr"/>
-      <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr"/>
-      <c r="J32" s="3" t="inlineStr"/>
-      <c r="K32" s="3" t="inlineStr"/>
-      <c r="L32" s="3" t="inlineStr"/>
-      <c r="M32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>boycott; political_or_religious_protest</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr"/>
+      <c r="I32" s="4" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr"/>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; Sweden; Islam</t>
+        </is>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>I hate this app and sweden</t>
+        </is>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr"/>
+      <c r="P32" s="4" t="inlineStr"/>
+      <c r="Q32" s="4" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1315,16 +2514,53 @@
       <c r="C33" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr"/>
-      <c r="J33" s="3" t="inlineStr"/>
-      <c r="K33" s="3" t="inlineStr"/>
-      <c r="L33" s="3" t="inlineStr"/>
-      <c r="M33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>app_stability; playback</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>bug_report</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr"/>
+      <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; app installation; playback</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>now I can't even open the app</t>
+        </is>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr"/>
+      <c r="P33" s="4" t="inlineStr"/>
+      <c r="Q33" s="4" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1340,16 +2576,53 @@
       <c r="C34" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D34" s="3" t="inlineStr"/>
-      <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="3" t="inlineStr"/>
-      <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr"/>
-      <c r="J34" s="3" t="inlineStr"/>
-      <c r="K34" s="3" t="inlineStr"/>
-      <c r="L34" s="3" t="inlineStr"/>
-      <c r="M34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>ads; audio_safety</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>safety_complaint</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr"/>
+      <c r="I34" s="4" t="inlineStr"/>
+      <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" s="4" t="inlineStr"/>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; ads; audio volume</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>my ears feel like they explode</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr"/>
+      <c r="P34" s="4" t="inlineStr"/>
+      <c r="Q34" s="4" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1365,16 +2638,53 @@
       <c r="C35" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr"/>
-      <c r="G35" s="3" t="inlineStr"/>
-      <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr"/>
-      <c r="J35" s="3" t="inlineStr"/>
-      <c r="K35" s="3" t="inlineStr"/>
-      <c r="L35" s="3" t="inlineStr"/>
-      <c r="M35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>unclear; promotion</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr"/>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr"/>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; subscription promotion</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>give me a free dollar to go with 3 months</t>
+        </is>
+      </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr"/>
+      <c r="P35" s="4" t="inlineStr"/>
+      <c r="Q35" s="4" t="inlineStr"/>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1390,16 +2700,53 @@
       <c r="C36" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D36" s="3" t="inlineStr"/>
-      <c r="E36" s="3" t="inlineStr"/>
-      <c r="F36" s="3" t="inlineStr"/>
-      <c r="G36" s="3" t="inlineStr"/>
-      <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr"/>
-      <c r="J36" s="3" t="inlineStr"/>
-      <c r="K36" s="3" t="inlineStr"/>
-      <c r="L36" s="3" t="inlineStr"/>
-      <c r="M36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr"/>
+      <c r="I36" s="4" t="inlineStr"/>
+      <c r="J36" s="4" t="inlineStr"/>
+      <c r="K36" s="4" t="inlineStr"/>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr"/>
+      <c r="P36" s="4" t="inlineStr"/>
+      <c r="Q36" s="4" t="inlineStr"/>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1415,16 +2762,53 @@
       <c r="C37" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D37" s="3" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr"/>
-      <c r="G37" s="3" t="inlineStr"/>
-      <c r="H37" s="3" t="inlineStr"/>
-      <c r="I37" s="3" t="inlineStr"/>
-      <c r="J37" s="3" t="inlineStr"/>
-      <c r="K37" s="3" t="inlineStr"/>
-      <c r="L37" s="3" t="inlineStr"/>
-      <c r="M37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>Good app!</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr"/>
+      <c r="P37" s="4" t="inlineStr"/>
+      <c r="Q37" s="4" t="inlineStr"/>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1440,16 +2824,53 @@
       <c r="C38" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D38" s="3" t="inlineStr"/>
-      <c r="E38" s="3" t="inlineStr"/>
-      <c r="F38" s="3" t="inlineStr"/>
-      <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="3" t="inlineStr"/>
-      <c r="J38" s="3" t="inlineStr"/>
-      <c r="K38" s="3" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr"/>
-      <c r="M38" s="3" t="inlineStr"/>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>ads</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr"/>
+      <c r="J38" s="4" t="inlineStr"/>
+      <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; advertising</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>very less advertising</t>
+        </is>
+      </c>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr"/>
+      <c r="P38" s="4" t="inlineStr"/>
+      <c r="Q38" s="4" t="inlineStr"/>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1465,16 +2886,53 @@
       <c r="C39" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr"/>
-      <c r="G39" s="3" t="inlineStr"/>
-      <c r="H39" s="3" t="inlineStr"/>
-      <c r="I39" s="3" t="inlineStr"/>
-      <c r="J39" s="3" t="inlineStr"/>
-      <c r="K39" s="3" t="inlineStr"/>
-      <c r="L39" s="3" t="inlineStr"/>
-      <c r="M39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>lyrics; playback_controls; app_update</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>bug_report</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; lyrics; playback controls</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>Lyrics not getting loaded</t>
+        </is>
+      </c>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr"/>
+      <c r="P39" s="4" t="inlineStr"/>
+      <c r="Q39" s="4" t="inlineStr"/>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1490,16 +2948,53 @@
       <c r="C40" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D40" s="3" t="inlineStr"/>
-      <c r="E40" s="3" t="inlineStr"/>
-      <c r="F40" s="3" t="inlineStr"/>
-      <c r="G40" s="3" t="inlineStr"/>
-      <c r="H40" s="3" t="inlineStr"/>
-      <c r="I40" s="3" t="inlineStr"/>
-      <c r="J40" s="3" t="inlineStr"/>
-      <c r="K40" s="3" t="inlineStr"/>
-      <c r="L40" s="3" t="inlineStr"/>
-      <c r="M40" s="3" t="inlineStr"/>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr"/>
+      <c r="J40" s="4" t="inlineStr"/>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>Phenomenal</t>
+        </is>
+      </c>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr"/>
+      <c r="P40" s="4" t="inlineStr"/>
+      <c r="Q40" s="4" t="inlineStr"/>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1515,16 +3010,53 @@
       <c r="C41" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr"/>
-      <c r="G41" s="3" t="inlineStr"/>
-      <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr"/>
-      <c r="J41" s="3" t="inlineStr"/>
-      <c r="K41" s="3" t="inlineStr"/>
-      <c r="L41" s="3" t="inlineStr"/>
-      <c r="M41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr"/>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="N41" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr"/>
+      <c r="P41" s="4" t="inlineStr"/>
+      <c r="Q41" s="4" t="inlineStr"/>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1542,16 +3074,53 @@
       <c r="C42" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D42" s="3" t="inlineStr"/>
-      <c r="E42" s="3" t="inlineStr"/>
-      <c r="F42" s="3" t="inlineStr"/>
-      <c r="G42" s="3" t="inlineStr"/>
-      <c r="H42" s="3" t="inlineStr"/>
-      <c r="I42" s="3" t="inlineStr"/>
-      <c r="J42" s="3" t="inlineStr"/>
-      <c r="K42" s="3" t="inlineStr"/>
-      <c r="L42" s="3" t="inlineStr"/>
-      <c r="M42" s="3" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>library_organization; feature_request</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>feature_request</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr"/>
+      <c r="J42" s="4" t="inlineStr"/>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; saved albums; artists; collections</t>
+        </is>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>ability to organize saved albums/artists into collections</t>
+        </is>
+      </c>
+      <c r="N42" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr"/>
+      <c r="P42" s="4" t="inlineStr"/>
+      <c r="Q42" s="4" t="inlineStr"/>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>NOT an exact substring of review_text</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1567,16 +3136,53 @@
       <c r="C43" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr"/>
-      <c r="G43" s="3" t="inlineStr"/>
-      <c r="H43" s="3" t="inlineStr"/>
-      <c r="I43" s="3" t="inlineStr"/>
-      <c r="J43" s="3" t="inlineStr"/>
-      <c r="K43" s="3" t="inlineStr"/>
-      <c r="L43" s="3" t="inlineStr"/>
-      <c r="M43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>general_dissatisfaction</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr"/>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>Worst application</t>
+        </is>
+      </c>
+      <c r="N43" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr"/>
+      <c r="P43" s="4" t="inlineStr"/>
+      <c r="Q43" s="4" t="inlineStr"/>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1592,16 +3198,53 @@
       <c r="C44" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D44" s="3" t="inlineStr"/>
-      <c r="E44" s="3" t="inlineStr"/>
-      <c r="F44" s="3" t="inlineStr"/>
-      <c r="G44" s="3" t="inlineStr"/>
-      <c r="H44" s="3" t="inlineStr"/>
-      <c r="I44" s="3" t="inlineStr"/>
-      <c r="J44" s="3" t="inlineStr"/>
-      <c r="K44" s="3" t="inlineStr"/>
-      <c r="L44" s="3" t="inlineStr"/>
-      <c r="M44" s="3" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>app_update; playback_controls</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="4" t="inlineStr"/>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; updates; playback controls</t>
+        </is>
+      </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>I can't even play the songs that I like</t>
+        </is>
+      </c>
+      <c r="N44" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr"/>
+      <c r="P44" s="4" t="inlineStr"/>
+      <c r="Q44" s="4" t="inlineStr"/>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1617,16 +3260,53 @@
       <c r="C45" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr"/>
-      <c r="G45" s="3" t="inlineStr"/>
-      <c r="H45" s="3" t="inlineStr"/>
-      <c r="I45" s="3" t="inlineStr"/>
-      <c r="J45" s="3" t="inlineStr"/>
-      <c r="K45" s="3" t="inlineStr"/>
-      <c r="L45" s="3" t="inlineStr"/>
-      <c r="M45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>music_discovery; recommendations</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; playlists; recommendations</t>
+        </is>
+      </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>it finds and play whatever music you want</t>
+        </is>
+      </c>
+      <c r="N45" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr"/>
+      <c r="P45" s="4" t="inlineStr"/>
+      <c r="Q45" s="4" t="inlineStr"/>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1642,16 +3322,53 @@
       <c r="C46" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D46" s="3" t="inlineStr"/>
-      <c r="E46" s="3" t="inlineStr"/>
-      <c r="F46" s="3" t="inlineStr"/>
-      <c r="G46" s="3" t="inlineStr"/>
-      <c r="H46" s="3" t="inlineStr"/>
-      <c r="I46" s="3" t="inlineStr"/>
-      <c r="J46" s="3" t="inlineStr"/>
-      <c r="K46" s="3" t="inlineStr"/>
-      <c r="L46" s="3" t="inlineStr"/>
-      <c r="M46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>offline_playback; subscription</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr"/>
+      <c r="J46" s="4" t="inlineStr"/>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; subscription; offline mode</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>unable to play in offline mode</t>
+        </is>
+      </c>
+      <c r="N46" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr"/>
+      <c r="P46" s="4" t="inlineStr"/>
+      <c r="Q46" s="4" t="inlineStr"/>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1667,16 +3384,53 @@
       <c r="C47" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D47" s="3" t="inlineStr"/>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr"/>
-      <c r="G47" s="3" t="inlineStr"/>
-      <c r="H47" s="3" t="inlineStr"/>
-      <c r="I47" s="3" t="inlineStr"/>
-      <c r="J47" s="3" t="inlineStr"/>
-      <c r="K47" s="3" t="inlineStr"/>
-      <c r="L47" s="3" t="inlineStr"/>
-      <c r="M47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>ads</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; ads</t>
+        </is>
+      </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>too much ad</t>
+        </is>
+      </c>
+      <c r="N47" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr"/>
+      <c r="P47" s="4" t="inlineStr"/>
+      <c r="Q47" s="4" t="inlineStr"/>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1692,16 +3446,53 @@
       <c r="C48" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D48" s="3" t="inlineStr"/>
-      <c r="E48" s="3" t="inlineStr"/>
-      <c r="F48" s="3" t="inlineStr"/>
-      <c r="G48" s="3" t="inlineStr"/>
-      <c r="H48" s="3" t="inlineStr"/>
-      <c r="I48" s="3" t="inlineStr"/>
-      <c r="J48" s="3" t="inlineStr"/>
-      <c r="K48" s="3" t="inlineStr"/>
-      <c r="L48" s="3" t="inlineStr"/>
-      <c r="M48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>pricing; ads; free_tier_limitations</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr"/>
+      <c r="I48" s="4" t="inlineStr"/>
+      <c r="J48" s="4" t="inlineStr"/>
+      <c r="K48" s="4" t="inlineStr"/>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; ads; subscription</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>free version is pretty much unusable with constant ads</t>
+        </is>
+      </c>
+      <c r="N48" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O48" s="4" t="inlineStr"/>
+      <c r="P48" s="4" t="inlineStr"/>
+      <c r="Q48" s="4" t="inlineStr"/>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1717,16 +3508,53 @@
       <c r="C49" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D49" s="3" t="inlineStr"/>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr"/>
-      <c r="G49" s="3" t="inlineStr"/>
-      <c r="H49" s="3" t="inlineStr"/>
-      <c r="I49" s="3" t="inlineStr"/>
-      <c r="J49" s="3" t="inlineStr"/>
-      <c r="K49" s="3" t="inlineStr"/>
-      <c r="L49" s="3" t="inlineStr"/>
-      <c r="M49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>app_update</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>complaint</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr"/>
+      <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="inlineStr"/>
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>Spotify; app updates</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>This update very bad for everyone</t>
+        </is>
+      </c>
+      <c r="N49" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O49" s="4" t="inlineStr"/>
+      <c r="P49" s="4" t="inlineStr"/>
+      <c r="Q49" s="4" t="inlineStr"/>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1742,16 +3570,53 @@
       <c r="C50" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D50" s="3" t="inlineStr"/>
-      <c r="E50" s="3" t="inlineStr"/>
-      <c r="F50" s="3" t="inlineStr"/>
-      <c r="G50" s="3" t="inlineStr"/>
-      <c r="H50" s="3" t="inlineStr"/>
-      <c r="I50" s="3" t="inlineStr"/>
-      <c r="J50" s="3" t="inlineStr"/>
-      <c r="K50" s="3" t="inlineStr"/>
-      <c r="L50" s="3" t="inlineStr"/>
-      <c r="M50" s="3" t="inlineStr"/>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>general_experience</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr"/>
+      <c r="I50" s="4" t="inlineStr"/>
+      <c r="J50" s="4" t="inlineStr"/>
+      <c r="K50" s="4" t="inlineStr"/>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M50" s="5" t="inlineStr">
+        <is>
+          <t>I'm loving the experience with the app</t>
+        </is>
+      </c>
+      <c r="N50" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O50" s="4" t="inlineStr"/>
+      <c r="P50" s="4" t="inlineStr"/>
+      <c r="Q50" s="4" t="inlineStr"/>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1767,35 +3632,73 @@
       <c r="C51" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D51" s="3" t="inlineStr"/>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr"/>
-      <c r="G51" s="3" t="inlineStr"/>
-      <c r="H51" s="3" t="inlineStr"/>
-      <c r="I51" s="3" t="inlineStr"/>
-      <c r="J51" s="3" t="inlineStr"/>
-      <c r="K51" s="3" t="inlineStr"/>
-      <c r="L51" s="3" t="inlineStr"/>
-      <c r="M51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>general_praise</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>praise</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr"/>
+      <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="inlineStr"/>
+      <c r="K51" s="4" t="inlineStr"/>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>best app ever</t>
+        </is>
+      </c>
+      <c r="N51" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O51" s="4" t="inlineStr"/>
+      <c r="P51" s="4" t="inlineStr"/>
+      <c r="Q51" s="4" t="inlineStr"/>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="0"/>
   <dataValidations count="6">
-    <dataValidation sqref="D2:D51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick from the list." promptTitle="topic" prompt="One primary topic (see Definitions tab)." type="list">
+    <dataValidation sqref="H2:H51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick from the list." promptTitle="topic" prompt="One primary topic (see Definitions tab)." type="list">
       <formula1>"access,usability,playback,downloads,catalog,billing,support,other"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick from the list." promptTitle="intent" prompt="Precedence: cancellation &gt; complaint &gt; request &gt; praise &gt; unclear." type="list">
+    <dataValidation sqref="I2:I51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick from the list." promptTitle="intent" prompt="Precedence: cancellation &gt; complaint &gt; request &gt; praise &gt; unclear." type="list">
       <formula1>"cancellation,complaint,request,praise,unclear"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick from the list." promptTitle="severity" prompt="1 no problem ... 5 serious financial/privacy/data harm." type="list">
+    <dataValidation sqref="J2:J51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick from the list." promptTitle="severity" prompt="1 no problem ... 5 serious financial/privacy/data harm." type="list">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick from the list." promptTitle="needs_review" prompt="TRUE if context is missing or the call is close." type="list">
+    <dataValidation sqref="N2:N51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick from the list." promptTitle="needs_review" prompt="TRUE if context is missing or the call is close." type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick from the list." promptTitle="ambiguous" prompt="TRUE if more than one label is defensible." type="list">
+    <dataValidation sqref="O2:O51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick from the list." promptTitle="ambiguous" prompt="TRUE if more than one label is defensible." type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" error="Sentiment must be between -1 and 1." promptTitle="sentiment" prompt="-1.0 (very negative) to 1.0 (very positive)." type="decimal" operator="between">
+    <dataValidation sqref="K2:K51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" error="Sentiment must be a number between -1 and 1." promptTitle="sentiment" prompt="-1.0 (very negative) to 1.0 (very positive)." type="decimal" operator="between">
       <formula1>-1</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -1810,7 +3713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1818,7 +3721,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>How to use</t>
         </is>
@@ -1826,98 +3729,110 @@
       <c r="B1" s="2" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Fill only the yellow cells on the Labels tab.</t>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Yellow cells</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Dropdowns: topic, intent, severity, needs_review, ambiguous. Sentiment accepts -1 to 1.</t>
+          <t>Fill these: topic, intent, severity, sentiment (dropdowns / -1..1), ambiguous, accepted_alternatives, notes.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Green cells</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Carried over from your own draft (evidence_quote, entities, needs_review). Editable; check them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Grey 'my_draft_*' columns</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Your own draft labels, locked for reference. They are not in the contract's label set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>check_quote_in_text</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Code check only: says whether your evidence_quote is an exact substring of review_text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Locked cells</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>The sheet is protected without a password (Review &gt; Unprotect Sheet) so review data and drafts are not edited by accident.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Feature terms the text explicitly names, separated by ';' (blank if none).</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>evidence_quote</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Copy an exact substring of review_text that supports the label.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>An exact substring of review_text that supports the label.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>accepted_alternatives</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Optional, e.g. topic=billing|usability; severity=2|3</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Save</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Keep this file as .xlsx; python -m pipeline eval golden reads it directly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Example format (made-up review, NOT one of the 50)</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>review_text</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>The app logs me out every morning and I can't get back in with my password.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>labels</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>topic=access; intent=complaint; severity=4; sentiment=-0.7; entities=login;password; evidence_quote=I can't get back in with my password; needs_review=FALSE; ambiguous=FALSE</t>
         </is>
       </c>
     </row>
@@ -1926,224 +3841,260 @@
       <c r="B11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Example format (made-up review, NOT one of the 50)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>review_text</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>The app logs me out every morning and I can't get back in with my password.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>labels</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>topic=access; intent=complaint; severity=4; sentiment=-0.7; entities=login;password; evidence_quote=I can't get back in with my password; needs_review=FALSE; ambiguous=FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>topic</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Definition (GRADING_CONTRACT.md)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>access</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Login, signup, password or account access</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>usability</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Navigation, controls, layout, queue/playlist management, ad interruptions</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>playback</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Playback failure, crashes, lag, connection failures, audio quality, resource use</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>downloads</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Downloading, saved music, offline listening, disappearing downloads</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>catalog</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Missing songs/artists, search/discovery, recommendations, lyrics availability</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>billing</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Price, charges, subscriptions, paywalls, premium entitlement; explicitly premium-only controls go here</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Contacting support and the support response</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>General praise/criticism, unrelated content, or no supported specific topic</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Topic tie rules</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Highest supported severity; on a tie, the first specific problem. Positive review: first specific praised feature; general praise is other. A paid-plan mention alone is not billing.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
-      <c r="B22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>intent</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>cancellation (explicitly leaving, uninstalling, cancelling, or threatening to) &gt; complaint (negative experience, incl. mixed) &gt; request (desired change, no reported failure) &gt; praise &gt; unclear. Bare boycott slogans and meaningless text are unclear. General 'bad app' is a complaint.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
-      <c r="B24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>No reported problem: praise, neutral/unclear content, or a pure feature request</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Dislike, generic criticism, minor annoyance, or cosmetic issue; no supported functional loss</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>A degraded or restricted function; some use or workaround remains</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>A clearly blocked core task, such as inability to log in or play music</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Explicit serious financial, privacy, or data harm; an expensive plan, a crash, or angry language alone is insufficient</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Cancellation intent does not raise severity. Missing context -&gt; needs_review; do not invent impact.</t>
         </is>

</xml_diff>